<commit_message>
new function in importer
</commit_message>
<xml_diff>
--- a/claude-finance-analyzer/importer/finance.xlsx
+++ b/claude-finance-analyzer/importer/finance.xlsx
@@ -25,7 +25,7 @@
     <t>Emittent</t>
   </si>
   <si>
-    <t xml:space="preserve">Buy in </t>
+    <t xml:space="preserve">Buyin </t>
   </si>
   <si>
     <t>Anzahl</t>
@@ -34,7 +34,7 @@
     <t>AI &amp; Big Data USD ( Acc)</t>
   </si>
   <si>
-    <t>XAIX</t>
+    <t>XAIX.DE</t>
   </si>
   <si>
     <t>Xtrackers</t>
@@ -43,7 +43,7 @@
     <t>Core MSCI World USD (Acc)</t>
   </si>
   <si>
-    <t>EUNL</t>
+    <t>EUNL.DE</t>
   </si>
   <si>
     <t>ishares</t>
@@ -52,7 +52,7 @@
     <t>S&amp;P 500 Information Tech USD (Acc)</t>
   </si>
   <si>
-    <t>QDVE</t>
+    <t>QDVE.DE</t>
   </si>
   <si>
     <t>NVIDIA</t>
@@ -76,7 +76,7 @@
     <t>Physical Swiss Gold USD</t>
   </si>
   <si>
-    <t>SGLD</t>
+    <t>SGLD.DE</t>
   </si>
   <si>
     <t>WisdomTree</t>
@@ -119,7 +119,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0&quot;€&quot;"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -130,6 +130,14 @@
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
     </font>
   </fonts>
   <fills count="2">
@@ -146,14 +154,20 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
@@ -406,7 +420,7 @@
       <c r="B2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="3">
         <v>1687.96</v>
       </c>
       <c r="D2" s="1" t="s">
@@ -423,7 +437,7 @@
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C3" s="1">
@@ -443,7 +457,7 @@
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="4" t="s">
         <v>13</v>
       </c>
       <c r="C4" s="1">
@@ -514,7 +528,7 @@
       <c r="A8" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="4" t="s">
         <v>21</v>
       </c>
       <c r="C8" s="1">
@@ -540,7 +554,7 @@
       <c r="C9" s="1">
         <v>87.25</v>
       </c>
-      <c r="E9" s="3">
+      <c r="E9" s="5">
         <v>90794.49</v>
       </c>
       <c r="F9" s="1">
@@ -619,6 +633,12 @@
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <hyperlinks>
+    <hyperlink r:id="rId1" ref="B2"/>
+    <hyperlink r:id="rId2" ref="B3"/>
+    <hyperlink r:id="rId3" ref="B4"/>
+    <hyperlink r:id="rId4" ref="B8"/>
+  </hyperlinks>
+  <drawing r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>